<commit_message>
Add granular per-day forward-return horizons (1-60 trading days) and --horizons CLI override. Finding: Reaccum-Reversal entry's optimal holding period is 4-7 trading days (win rate peaks 67.5% at day4, avg return peaks 1.48% at day7); edge decays steadily beyond day 10-15, down to 47-53% win rate by day 20-30. Documented in README.
</commit_message>
<xml_diff>
--- a/results/backtest_simple.xlsx
+++ b/results/backtest_simple.xlsx
@@ -546,49 +546,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TORNTPHARM.NS</t>
+          <t>SIEMENS.NS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SIEMENS.NS</t>
+          <t>TORNTPHARM.NS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">

</xml_diff>

<commit_message>
Add composite setup-quality scoring (A/B/C/D grades, 0-100 score) combining confluence (40pts), structure cleanliness/num reversals (20pts), volatility contraction (15pts), re-accumulation duration fit (15pts), and stage maturity (10pts).
Wired into: live scanner output + Telegram alerts, backtest Live Signals Now sheet, backtest_simple.xlsx (new 'Setup Quality' 6th column, color-coded), and backtest_results.xlsx. Historical rows scored as-of the signal date (no look-ahead bias) vs live rows scored as-of today.

Validated: PGIL=A(88), AUBANK=B(71) live; POWERGRID's FRESH_REVERSAL correctly flagged D(33.9, weak) vs ABB's B(69.1) despite same stage. Grade distribution across 175 backtest rows: 74 A / 62 B / 29 C / 10 D - meaningful spread, not degenerate.
</commit_message>
<xml_diff>
--- a/results/backtest_simple.xlsx
+++ b/results/backtest_simple.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -44,6 +44,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -73,6 +97,10 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -150,14 +178,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacktestResults" displayName="BacktestResults" ref="A1:E176" headerRowCount="1">
-  <autoFilter ref="A1:E176"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacktestResults" displayName="BacktestResults" ref="A1:F176" headerRowCount="1">
+  <autoFilter ref="A1:F176"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="Symbol"/>
     <tableColumn id="2" name="BOS1 Breakout Date"/>
     <tableColumn id="3" name="Retest Date"/>
     <tableColumn id="4" name="Re-Accumulation Date"/>
     <tableColumn id="5" name="Reversal Date"/>
+    <tableColumn id="6" name="Setup Quality"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -452,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E176"/>
+  <dimension ref="A1:F176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -460,6 +489,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,301 +518,361 @@
           <t>Reversal Date</t>
         </is>
       </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Setup Quality</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BIOCON.NS</t>
+          <t>ABB.NS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABB.NS</t>
+          <t>SIEMENS.NS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SIEMENS.NS</t>
+          <t>TORNTPHARM.NS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TORNTPHARM.NS</t>
+          <t>BAJFINANCE.NS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BAJFINANCE.NS</t>
+          <t>PIDILITIND.NS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GRASIM.NS</t>
+          <t>LUPIN.NS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>LUPIN.NS</t>
+          <t>AUROPHARMA.NS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AUROPHARMA.NS</t>
+          <t>PGIL.NS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PGIL.NS</t>
+          <t>MOTHERSON.NS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MOTHERSON.NS</t>
+          <t>BHARATFORG.NS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BHARATFORG.NS</t>
+          <t>GRASIM.NS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
         </is>
       </c>
     </row>
@@ -812,6 +902,11 @@
           <t>2026-07-27</t>
         </is>
       </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -839,193 +934,233 @@
           <t>2026-07-27</t>
         </is>
       </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PIDILITIND.NS</t>
+          <t>AUBANK.NS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AUBANK.NS</t>
+          <t>NESTLEIND.NS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NESTLEIND.NS</t>
+          <t>INDUSINDBK.NS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>INDUSINDBK.NS</t>
+          <t>POLYCAB.NS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>POLYCAB.NS</t>
+          <t>IPCALAB.NS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IPCALAB.NS</t>
+          <t>ADANIENT.NS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ADANIENT.NS</t>
+          <t>BIOCON.NS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
         </is>
       </c>
     </row>
@@ -1055,6 +1190,11 @@
           <t>2026-06-30</t>
         </is>
       </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1082,6 +1222,11 @@
           <t>2026-06-29</t>
         </is>
       </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1109,6 +1254,11 @@
           <t>2026-06-18</t>
         </is>
       </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1136,6 +1286,11 @@
           <t>2026-06-17</t>
         </is>
       </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1163,6 +1318,11 @@
           <t>2026-06-15</t>
         </is>
       </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1190,6 +1350,11 @@
           <t>2026-06-15</t>
         </is>
       </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1217,6 +1382,11 @@
           <t>2026-06-12</t>
         </is>
       </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1244,6 +1414,11 @@
           <t>2026-06-12</t>
         </is>
       </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1271,6 +1446,11 @@
           <t>2026-06-12</t>
         </is>
       </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1298,6 +1478,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1325,6 +1510,11 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1352,6 +1542,11 @@
           <t>2026-06-04</t>
         </is>
       </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1379,6 +1574,11 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1406,6 +1606,11 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1433,6 +1638,11 @@
           <t>2026-06-03</t>
         </is>
       </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1460,6 +1670,11 @@
           <t>2026-05-27</t>
         </is>
       </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1487,6 +1702,11 @@
           <t>2026-05-27</t>
         </is>
       </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1514,6 +1734,11 @@
           <t>2026-05-14</t>
         </is>
       </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1541,6 +1766,11 @@
           <t>2026-05-07</t>
         </is>
       </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1568,6 +1798,11 @@
           <t>2026-05-06</t>
         </is>
       </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1595,6 +1830,11 @@
           <t>2026-05-04</t>
         </is>
       </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1622,6 +1862,11 @@
           <t>2026-04-08</t>
         </is>
       </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1649,6 +1894,11 @@
           <t>2026-04-07</t>
         </is>
       </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1676,6 +1926,11 @@
           <t>2026-04-06</t>
         </is>
       </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1703,6 +1958,11 @@
           <t>2026-04-02</t>
         </is>
       </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1730,6 +1990,11 @@
           <t>2026-03-30</t>
         </is>
       </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1757,6 +2022,11 @@
           <t>2026-03-24</t>
         </is>
       </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1784,6 +2054,11 @@
           <t>2026-03-20</t>
         </is>
       </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1811,6 +2086,11 @@
           <t>2026-03-17</t>
         </is>
       </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1838,6 +2118,11 @@
           <t>2026-03-17</t>
         </is>
       </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1865,6 +2150,11 @@
           <t>2026-03-10</t>
         </is>
       </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1892,6 +2182,11 @@
           <t>2026-03-10</t>
         </is>
       </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1919,6 +2214,11 @@
           <t>2026-03-10</t>
         </is>
       </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1946,6 +2246,11 @@
           <t>2026-03-10</t>
         </is>
       </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1973,6 +2278,11 @@
           <t>2026-03-05</t>
         </is>
       </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2000,6 +2310,11 @@
           <t>2026-03-05</t>
         </is>
       </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2027,6 +2342,11 @@
           <t>2026-02-20</t>
         </is>
       </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2054,6 +2374,11 @@
           <t>2026-02-19</t>
         </is>
       </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2081,6 +2406,11 @@
           <t>2026-02-18</t>
         </is>
       </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2108,6 +2438,11 @@
           <t>2026-02-17</t>
         </is>
       </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2135,6 +2470,11 @@
           <t>2026-02-17</t>
         </is>
       </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2162,6 +2502,11 @@
           <t>2026-02-17</t>
         </is>
       </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2189,6 +2534,11 @@
           <t>2026-02-17</t>
         </is>
       </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2216,6 +2566,11 @@
           <t>2026-02-16</t>
         </is>
       </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2243,6 +2598,11 @@
           <t>2026-02-16</t>
         </is>
       </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2270,6 +2630,11 @@
           <t>2026-02-16</t>
         </is>
       </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2297,6 +2662,11 @@
           <t>2026-02-06</t>
         </is>
       </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2324,6 +2694,11 @@
           <t>2026-02-04</t>
         </is>
       </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2351,6 +2726,11 @@
           <t>2026-02-04</t>
         </is>
       </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2378,6 +2758,11 @@
           <t>2026-02-04</t>
         </is>
       </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2405,6 +2790,11 @@
           <t>2026-02-03</t>
         </is>
       </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2432,6 +2822,11 @@
           <t>2026-02-03</t>
         </is>
       </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2459,6 +2854,11 @@
           <t>2026-02-03</t>
         </is>
       </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2486,6 +2886,11 @@
           <t>2026-01-29</t>
         </is>
       </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2513,6 +2918,11 @@
           <t>2026-01-28</t>
         </is>
       </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2540,6 +2950,11 @@
           <t>2026-01-28</t>
         </is>
       </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2567,6 +2982,11 @@
           <t>2026-01-28</t>
         </is>
       </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2594,6 +3014,11 @@
           <t>2026-01-28</t>
         </is>
       </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2621,6 +3046,11 @@
           <t>2026-01-28</t>
         </is>
       </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2648,6 +3078,11 @@
           <t>2026-01-27</t>
         </is>
       </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2675,6 +3110,11 @@
           <t>2026-01-22</t>
         </is>
       </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2702,6 +3142,11 @@
           <t>2026-01-22</t>
         </is>
       </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2729,6 +3174,11 @@
           <t>2026-01-22</t>
         </is>
       </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2756,6 +3206,11 @@
           <t>2026-01-16</t>
         </is>
       </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2783,6 +3238,11 @@
           <t>2026-01-16</t>
         </is>
       </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2810,6 +3270,11 @@
           <t>2026-01-16</t>
         </is>
       </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2837,6 +3302,11 @@
           <t>2026-01-13</t>
         </is>
       </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2864,6 +3334,11 @@
           <t>2026-01-12</t>
         </is>
       </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2891,6 +3366,11 @@
           <t>2026-01-12</t>
         </is>
       </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2918,6 +3398,11 @@
           <t>2026-01-07</t>
         </is>
       </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2945,6 +3430,11 @@
           <t>2026-01-05</t>
         </is>
       </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2972,6 +3462,11 @@
           <t>2026-01-02</t>
         </is>
       </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2999,6 +3494,11 @@
           <t>2026-01-02</t>
         </is>
       </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3026,6 +3526,11 @@
           <t>2026-01-01</t>
         </is>
       </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3053,6 +3558,11 @@
           <t>2026-01-01</t>
         </is>
       </c>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3080,6 +3590,11 @@
           <t>2025-12-31</t>
         </is>
       </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3107,6 +3622,11 @@
           <t>2025-12-31</t>
         </is>
       </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3134,6 +3654,11 @@
           <t>2025-12-31</t>
         </is>
       </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3161,6 +3686,11 @@
           <t>2025-12-31</t>
         </is>
       </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3188,6 +3718,11 @@
           <t>2025-12-31</t>
         </is>
       </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3215,6 +3750,11 @@
           <t>2025-12-30</t>
         </is>
       </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3242,6 +3782,11 @@
           <t>2025-12-24</t>
         </is>
       </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3269,6 +3814,11 @@
           <t>2025-12-22</t>
         </is>
       </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3296,6 +3846,11 @@
           <t>2025-12-19</t>
         </is>
       </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -3323,6 +3878,11 @@
           <t>2025-12-19</t>
         </is>
       </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3350,6 +3910,11 @@
           <t>2025-12-15</t>
         </is>
       </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -3377,6 +3942,11 @@
           <t>2025-12-15</t>
         </is>
       </c>
+      <c r="F108" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3404,6 +3974,11 @@
           <t>2025-12-12</t>
         </is>
       </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3431,6 +4006,11 @@
           <t>2025-12-12</t>
         </is>
       </c>
+      <c r="F110" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3458,6 +4038,11 @@
           <t>2025-12-11</t>
         </is>
       </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3485,6 +4070,11 @@
           <t>2025-12-11</t>
         </is>
       </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -3512,6 +4102,11 @@
           <t>2025-12-05</t>
         </is>
       </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -3539,6 +4134,11 @@
           <t>2025-11-27</t>
         </is>
       </c>
+      <c r="F114" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -3566,6 +4166,11 @@
           <t>2025-11-26</t>
         </is>
       </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -3593,6 +4198,11 @@
           <t>2025-11-26</t>
         </is>
       </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -3620,6 +4230,11 @@
           <t>2025-11-25</t>
         </is>
       </c>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -3647,6 +4262,11 @@
           <t>2025-11-25</t>
         </is>
       </c>
+      <c r="F118" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -3674,6 +4294,11 @@
           <t>2025-11-20</t>
         </is>
       </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -3701,6 +4326,11 @@
           <t>2025-11-19</t>
         </is>
       </c>
+      <c r="F120" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -3728,6 +4358,11 @@
           <t>2025-11-13</t>
         </is>
       </c>
+      <c r="F121" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -3755,6 +4390,11 @@
           <t>2025-11-12</t>
         </is>
       </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -3782,6 +4422,11 @@
           <t>2025-11-10</t>
         </is>
       </c>
+      <c r="F123" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -3809,6 +4454,11 @@
           <t>2025-11-10</t>
         </is>
       </c>
+      <c r="F124" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -3836,6 +4486,11 @@
           <t>2025-11-06</t>
         </is>
       </c>
+      <c r="F125" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -3863,6 +4518,11 @@
           <t>2025-11-04</t>
         </is>
       </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -3890,6 +4550,11 @@
           <t>2025-10-29</t>
         </is>
       </c>
+      <c r="F127" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -3917,6 +4582,11 @@
           <t>2025-10-28</t>
         </is>
       </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -3944,6 +4614,11 @@
           <t>2025-10-27</t>
         </is>
       </c>
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -3971,6 +4646,11 @@
           <t>2025-10-20</t>
         </is>
       </c>
+      <c r="F130" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -3998,6 +4678,11 @@
           <t>2025-10-20</t>
         </is>
       </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4025,6 +4710,11 @@
           <t>2025-10-20</t>
         </is>
       </c>
+      <c r="F132" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4052,6 +4742,11 @@
           <t>2025-10-20</t>
         </is>
       </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4079,6 +4774,11 @@
           <t>2025-10-16</t>
         </is>
       </c>
+      <c r="F134" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4106,6 +4806,11 @@
           <t>2025-10-15</t>
         </is>
       </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -4133,6 +4838,11 @@
           <t>2025-10-07</t>
         </is>
       </c>
+      <c r="F136" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -4160,6 +4870,11 @@
           <t>2025-10-06</t>
         </is>
       </c>
+      <c r="F137" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -4187,6 +4902,11 @@
           <t>2025-10-06</t>
         </is>
       </c>
+      <c r="F138" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -4214,6 +4934,11 @@
           <t>2025-10-03</t>
         </is>
       </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4241,6 +4966,11 @@
           <t>2025-10-01</t>
         </is>
       </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -4268,6 +4998,11 @@
           <t>2025-10-01</t>
         </is>
       </c>
+      <c r="F141" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -4295,6 +5030,11 @@
           <t>2025-09-29</t>
         </is>
       </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -4322,6 +5062,11 @@
           <t>2025-09-18</t>
         </is>
       </c>
+      <c r="F143" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -4349,6 +5094,11 @@
           <t>2025-09-16</t>
         </is>
       </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -4376,6 +5126,11 @@
           <t>2025-09-11</t>
         </is>
       </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -4403,6 +5158,11 @@
           <t>2025-09-10</t>
         </is>
       </c>
+      <c r="F146" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -4430,6 +5190,11 @@
           <t>2025-09-02</t>
         </is>
       </c>
+      <c r="F147" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -4457,6 +5222,11 @@
           <t>2025-09-01</t>
         </is>
       </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -4484,6 +5254,11 @@
           <t>2025-09-01</t>
         </is>
       </c>
+      <c r="F149" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -4511,6 +5286,11 @@
           <t>2025-09-01</t>
         </is>
       </c>
+      <c r="F150" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -4538,6 +5318,11 @@
           <t>2025-08-18</t>
         </is>
       </c>
+      <c r="F151" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -4565,6 +5350,11 @@
           <t>2025-08-18</t>
         </is>
       </c>
+      <c r="F152" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -4592,6 +5382,11 @@
           <t>2025-08-14</t>
         </is>
       </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -4619,6 +5414,11 @@
           <t>2025-08-13</t>
         </is>
       </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -4646,6 +5446,11 @@
           <t>2025-08-13</t>
         </is>
       </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -4673,6 +5478,11 @@
           <t>2025-08-11</t>
         </is>
       </c>
+      <c r="F156" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -4700,6 +5510,11 @@
           <t>2025-08-07</t>
         </is>
       </c>
+      <c r="F157" s="6" t="inlineStr">
+        <is>
+          <t>D - Weak / Low-Quality</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -4727,6 +5542,11 @@
           <t>2025-08-04</t>
         </is>
       </c>
+      <c r="F158" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -4754,6 +5574,11 @@
           <t>2025-07-16</t>
         </is>
       </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -4781,6 +5606,11 @@
           <t>2025-07-15</t>
         </is>
       </c>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -4808,6 +5638,11 @@
           <t>2025-07-07</t>
         </is>
       </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -4835,6 +5670,11 @@
           <t>2025-06-25</t>
         </is>
       </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -4862,6 +5702,11 @@
           <t>2025-06-23</t>
         </is>
       </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -4889,6 +5734,11 @@
           <t>2025-06-23</t>
         </is>
       </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -4916,6 +5766,11 @@
           <t>2025-06-16</t>
         </is>
       </c>
+      <c r="F165" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -4943,6 +5798,11 @@
           <t>2025-06-16</t>
         </is>
       </c>
+      <c r="F166" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -4970,6 +5830,11 @@
           <t>2025-06-16</t>
         </is>
       </c>
+      <c r="F167" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -4997,6 +5862,11 @@
           <t>2025-06-16</t>
         </is>
       </c>
+      <c r="F168" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -5024,6 +5894,11 @@
           <t>2025-06-16</t>
         </is>
       </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -5051,6 +5926,11 @@
           <t>2025-06-06</t>
         </is>
       </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -5078,6 +5958,11 @@
           <t>2025-06-05</t>
         </is>
       </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -5105,6 +5990,11 @@
           <t>2025-06-04</t>
         </is>
       </c>
+      <c r="F172" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -5132,6 +6022,11 @@
           <t>2025-06-03</t>
         </is>
       </c>
+      <c r="F173" s="4" t="inlineStr">
+        <is>
+          <t>B - Good Setup</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -5159,6 +6054,11 @@
           <t>2025-05-23</t>
         </is>
       </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -5186,6 +6086,11 @@
           <t>2025-05-12</t>
         </is>
       </c>
+      <c r="F175" s="5" t="inlineStr">
+        <is>
+          <t>C - Moderate / Watch</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -5211,6 +6116,11 @@
       <c r="E176" t="inlineStr">
         <is>
           <t>2025-04-08</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>A - High-Quality Setup</t>
         </is>
       </c>
     </row>

</xml_diff>